<commit_message>
Updated DACD fixing TREND function
</commit_message>
<xml_diff>
--- a/InputData/geoeng/DACD/Direct Air Capture Data.xlsx
+++ b/InputData/geoeng/DACD/Direct Air Capture Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shigu\Documents\_swj\_Talanoa\CPSA Fletcher\dados\InputData (BR) 2024\d11 geoeng\DACD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tfranc03/Developer/eps-brazil-cpl/InputData/geoeng/DACD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9E7CF6-887A-4EB0-B50E-18D492E02955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26ED1147-E732-BD46-BE72-AF90FF439347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5604" yWindow="2160" windowWidth="17220" windowHeight="9912" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-45180" yWindow="2940" windowWidth="31000" windowHeight="21780" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,16 @@
     <sheet name="DACD-energyintensity" sheetId="5" r:id="rId5"/>
     <sheet name="DACD-capex" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'DACD-potential'!$A$1</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'DACD-potential'!$A$2</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'DACD-potential'!$B$1:$AI$1</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'DACD-potential'!$B$2:$AI$2</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'DACD-potential'!$A$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">'DACD-potential'!$A$2</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">'DACD-potential'!$B$1:$AI$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">'DACD-potential'!$B$2:$AI$2</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,6 +49,28 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="110">
   <si>
@@ -168,9 +200,6 @@
     <t>Global DAC Potential</t>
   </si>
   <si>
-    <t>U.S. DAC potential</t>
-  </si>
-  <si>
     <t>Converting to metric tons:</t>
   </si>
   <si>
@@ -370,16 +399,20 @@
   </si>
   <si>
     <t>Brazil GDP share</t>
+  </si>
+  <si>
+    <t>Brazil DAC potential</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000E+00"/>
+    <numFmt numFmtId="169" formatCode="0.00000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -467,7 +500,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -495,11 +528,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -512,6 +546,1031 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'DACD-potential'!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>DAC Potential</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'DACD-potential'!$B$1:$AI$1</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>2017</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2018</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2021</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2022</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2025</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2027</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2028</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2029</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2030</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2031</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2032</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2033</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2034</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2035</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2036</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2037</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2038</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2039</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2040</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2041</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2042</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2043</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2044</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2045</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2046</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2047</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2048</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2049</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2050</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'DACD-potential'!$B$2:$AI$2</c:f>
+              <c:numCache>
+                <c:formatCode>0.000E+00</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1833928.571428299</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3667857.1428565979</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>5501785.7142853737</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>7335714.2857141495</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>9169642.8571424484</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-87C2-4E42-AF44-665630252977}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="155716672"/>
+        <c:axId val="155718464"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="155716672"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="155718464"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="155718464"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.000E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="155716672"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -663,6 +1722,47 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1464469</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>112713</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>55563</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{492A2AD7-C5A2-9523-EE98-AB7EFE572C25}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -932,153 +2032,153 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.21875" customWidth="1"/>
-    <col min="2" max="2" width="47.21875" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" customWidth="1"/>
+    <col min="2" max="2" width="47.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7" s="6">
         <v>2019</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B9" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B11" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B16" s="6">
         <v>2023</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B18" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B18" s="5" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1095,93 +2195,93 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C706B8D-FB10-40CA-B025-270C2E82347D}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.21875" customWidth="1"/>
-    <col min="4" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.1640625" customWidth="1"/>
+    <col min="4" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B1">
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
         <v>86</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
-        <v>87</v>
       </c>
       <c r="B3">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B4">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B6">
         <f>B3/B1*1.25</f>
         <v>8.9285714285714274E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B7">
         <f>B4/B1*1.25</f>
         <v>0.3571428571428571</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B16">
         <v>2020</v>
       </c>
@@ -1195,9 +2295,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1224,60 +2324,60 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H105"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.21875" customWidth="1"/>
-    <col min="2" max="8" width="11.44140625" customWidth="1"/>
+    <col min="1" max="1" width="33.1640625" customWidth="1"/>
+    <col min="2" max="8" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
@@ -1286,7 +2386,7 @@
       <c r="F12" s="14"/>
       <c r="G12" s="14"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>6</v>
       </c>
@@ -1297,7 +2397,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1308,7 +2408,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
@@ -1319,7 +2419,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1330,12 +2430,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
@@ -1346,7 +2446,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>1</v>
       </c>
@@ -1357,7 +2457,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>2</v>
       </c>
@@ -1368,17 +2468,17 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>9</v>
       </c>
@@ -1389,7 +2489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>1</v>
       </c>
@@ -1400,7 +2500,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>2</v>
       </c>
@@ -1411,34 +2511,34 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B30" s="18">
         <v>0.67</v>
       </c>
       <c r="D30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="1"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>9</v>
       </c>
@@ -1449,7 +2549,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>1</v>
       </c>
@@ -1462,7 +2562,7 @@
         <v>2.3759999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>2</v>
       </c>
@@ -1475,27 +2575,27 @@
         <v>1.452</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
         <v>41</v>
       </c>
@@ -1507,27 +2607,27 @@
       <c r="G62" s="9"/>
       <c r="H62" s="9"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B68">
         <v>2045</v>
       </c>
@@ -1550,7 +2650,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>29</v>
       </c>
@@ -1576,7 +2676,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>30</v>
       </c>
@@ -1602,7 +2702,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>31</v>
       </c>
@@ -1610,7 +2710,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B74">
         <v>2045</v>
       </c>
@@ -1633,7 +2733,7 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>32</v>
       </c>
@@ -1659,7 +2759,7 @@
         <v>27.071428571428573</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>33</v>
       </c>
@@ -1685,29 +2785,29 @@
         <v>2.8571428571428568</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B83">
         <v>2.0539999999999998</v>
@@ -1719,7 +2819,7 @@
         <v>2017</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>38</v>
       </c>
@@ -1733,18 +2833,18 @@
         <v>2017</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B85" s="8">
         <f>B83/B84</f>
         <v>2.5674999999999996E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
-        <v>42</v>
+        <v>109</v>
       </c>
       <c r="B87" s="9"/>
       <c r="C87" s="9"/>
@@ -1754,7 +2854,7 @@
       <c r="G87" s="9"/>
       <c r="H87" s="9"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B88">
         <v>2045</v>
       </c>
@@ -1777,78 +2877,78 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>32</v>
       </c>
-      <c r="B89">
+      <c r="B89" s="19">
         <f>B75*$B$85</f>
         <v>0</v>
       </c>
-      <c r="C89" s="7">
+      <c r="C89" s="19">
         <f t="shared" ref="C89:H90" si="0">C75*$B$85</f>
         <v>9.1696428571428554E-3</v>
       </c>
-      <c r="D89" s="7">
+      <c r="D89" s="19">
         <f t="shared" si="0"/>
         <v>3.6678571428571421E-2</v>
       </c>
-      <c r="E89" s="7">
+      <c r="E89" s="19">
         <f t="shared" si="0"/>
         <v>0.2237392857142857</v>
       </c>
-      <c r="F89" s="7">
+      <c r="F89" s="19">
         <f t="shared" si="0"/>
         <v>0.71156428571428565</v>
       </c>
-      <c r="G89" s="7">
+      <c r="G89" s="19">
         <f t="shared" si="0"/>
         <v>0.70422857142857131</v>
       </c>
-      <c r="H89" s="7">
+      <c r="H89" s="19">
         <f t="shared" si="0"/>
         <v>0.69505892857142848</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>33</v>
       </c>
-      <c r="B90">
+      <c r="B90" s="19">
         <f>B76*$B$85</f>
         <v>0</v>
       </c>
-      <c r="C90">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D90">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E90" s="7">
+      <c r="C90" s="19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D90" s="19">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E90" s="19">
         <f t="shared" si="0"/>
         <v>9.1696428571428554E-3</v>
       </c>
-      <c r="F90" s="7">
+      <c r="F90" s="19">
         <f t="shared" si="0"/>
         <v>5.5017857142857132E-2</v>
       </c>
-      <c r="G90" s="7">
+      <c r="G90" s="19">
         <f t="shared" si="0"/>
         <v>6.4187499999999995E-2</v>
       </c>
-      <c r="H90" s="7">
+      <c r="H90" s="19">
         <f t="shared" si="0"/>
         <v>7.3357142857142843E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B93">
         <v>2045</v>
       </c>
@@ -1871,9 +2971,9 @@
         <v>2100</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B94" s="10">
         <f>B89*10^9</f>
@@ -1904,9 +3004,9 @@
         <v>695058928.57142854</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B95" s="10">
         <f>B90*10^9</f>
@@ -1937,42 +3037,42 @@
         <v>73357142.857142836</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
-        <v>52</v>
       </c>
       <c r="B103">
         <v>947086</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1988,18 +3088,19 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AI2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.77734375" customWidth="1"/>
-    <col min="2" max="2" width="9.21875" customWidth="1"/>
+    <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" customWidth="1"/>
     <col min="3" max="24" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="35" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="26" max="29" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1">
         <v>2017</v>
@@ -2104,9 +3205,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2" s="16">
         <v>0</v>
@@ -2192,33 +3293,30 @@
       <c r="AC2" s="16">
         <v>0</v>
       </c>
-      <c r="AD2">
-        <f>TREND(Data!$C$94:$D$94,Data!$C$93:$D$93,AD$1)</f>
-        <v>-4584821.4285707474</v>
-      </c>
-      <c r="AE2">
-        <f>TREND(Data!$C$94:$D$94,Data!$C$93:$D$93,AE$1)</f>
-        <v>-1833928.571428299</v>
-      </c>
-      <c r="AF2">
-        <f>TREND(Data!$C$94:$D$94,Data!$C$93:$D$93,AF$1)</f>
-        <v>916964.28571510315</v>
-      </c>
-      <c r="AG2">
-        <f>TREND(Data!$C$94:$D$94,Data!$C$93:$D$93,AG$1)</f>
-        <v>3667857.1428575516</v>
-      </c>
-      <c r="AH2">
-        <f>TREND(Data!$C$94:$D$94,Data!$C$93:$D$93,AH$1)</f>
-        <v>6418750</v>
-      </c>
-      <c r="AI2">
-        <f>TREND(Data!$C$94:$D$94,Data!$C$93:$D$93,AI$1)</f>
-        <v>9169642.8571434021</v>
+      <c r="AD2" s="16">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="16" cm="1">
+        <f t="array" ref="AE2:AI2">TREND(Data!$B$94:$C$94,Data!$B$93:$C$93,AE1:AI1)</f>
+        <v>1833928.571428299</v>
+      </c>
+      <c r="AF2" s="16">
+        <v>3667857.1428565979</v>
+      </c>
+      <c r="AG2" s="16">
+        <v>5501785.7142853737</v>
+      </c>
+      <c r="AH2" s="16">
+        <v>7335714.2857141495</v>
+      </c>
+      <c r="AI2" s="16">
+        <v>9169642.8571424484</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2228,15 +3326,15 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AI11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="9.21875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1">
         <v>2017</v>
@@ -2341,9 +3439,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" s="12">
         <f>Data!$C$20*Data!$C$103</f>
@@ -2482,149 +3580,149 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S3" s="12">
+        <f t="shared" ref="D3:AI10" si="2">$B3</f>
+        <v>0</v>
+      </c>
+      <c r="T3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AG3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI3" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>58</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="N3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="P3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Q3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="S3" s="12">
-        <f t="shared" ref="D2:AI10" si="2">$B3</f>
-        <v>0</v>
-      </c>
-      <c r="T3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI3" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>59</v>
       </c>
       <c r="B4" s="12">
         <f>Data!$C$26*Data!$B$103</f>
@@ -2763,709 +3861,709 @@
         <v>6819019.2000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>60</v>
       </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI5" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AG6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI6" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>61</v>
       </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI6" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AG7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI7" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>62</v>
       </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI7" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AG8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI8" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>63</v>
       </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI8" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AA9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AG9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI9" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>64</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="N9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AC9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AD9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AE9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AG9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AH9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AI9" s="12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>65</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -3603,9 +4701,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -3754,15 +4852,15 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AI2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="9.21875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B1">
         <v>2017</v>
@@ -3867,9 +4965,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" s="12">
         <f>Data!B14</f>

</xml_diff>